<commit_message>
Stálá ID zjištění; text analytika k Ekonomickému profilu a opravy; pilot schválen
- Zjištění mají stálé ID odvozené z typu a obsahu (ZXX-XXXX, bez číslic), ne
  z pořadí; pořadí podle síly je v poli „poradi“.
- V reporty/vyklad/F__CZ051__2026-09-15.md mechanicky zaměněno 18 odkazů Zxx
  za stálá ID (povoleno zadáním); jiná slova beze změny.
- Opravy textu analytika podle zadání (Shrnutí, Postavení území, Zaměstnanost
  a mzdy) a nový text oddílu Ekonomický profil; pilot vysázen s --vyklad-schvalen.
- Testy: stálá ID, každý odkaz ve výkladu existuje v zjisteni.json.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CRXzTFf4VAheMPr1kwwKwf
</commit_message>
<xml_diff>
--- a/reporty/ukazky/F__CZ051__2026-09-15/priloha.xlsx
+++ b/reporty/ukazky/F__CZ051__2026-09-15/priloha.xlsx
@@ -5684,7 +5684,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Z01</t>
+          <t>ZTR-IMTV</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Z02</t>
+          <t>ZTR-CISP</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -5742,7 +5742,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Z03</t>
+          <t>ZTR-LQXC</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Z04</t>
+          <t>ZTR-YGEL</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -5800,7 +5800,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Z05</t>
+          <t>ZPO-QDHA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -5826,7 +5826,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Z06</t>
+          <t>ZUZ-EGWN</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -5855,7 +5855,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Z07</t>
+          <t>ZOD-SXHQ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -5884,7 +5884,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Z08</t>
+          <t>ZOD-SRRX</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -5913,7 +5913,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Z09</t>
+          <t>ZOD-CAID</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -5942,7 +5942,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Z10</t>
+          <t>ZUZ-OWLP</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Z11</t>
+          <t>ZOD-PUOD</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Z12</t>
+          <t>ZOD-YZQO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -6029,7 +6029,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Z13</t>
+          <t>ZUZ-ADGK</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -6058,7 +6058,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Z14</t>
+          <t>ZMZ-ULLF</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Z15</t>
+          <t>ZUZ-DHYT</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -6116,7 +6116,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Z16</t>
+          <t>ZUZ-OXBR</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -6145,7 +6145,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Z17</t>
+          <t>ZOD-TOQY</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -6174,7 +6174,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Z18</t>
+          <t>ZOD-NDPG</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Z19</t>
+          <t>ZUZ-CLRE</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -6232,7 +6232,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Z20</t>
+          <t>ZUZ-HFUA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -6261,7 +6261,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Z21</t>
+          <t>ZOD-DWBZ</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -6290,7 +6290,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Z22</t>
+          <t>ZTR-RMDL</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -6319,7 +6319,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Z23</t>
+          <t>ZOD-SMOT</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -6348,7 +6348,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Z24</t>
+          <t>ZOD-KHDN</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -6377,7 +6377,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Z25</t>
+          <t>ZMZ-TZVU</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Z26</t>
+          <t>ZAK-CUQD</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -6435,7 +6435,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Z27</t>
+          <t>ZOD-DKSF</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Z28</t>
+          <t>ZOD-YNST</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -6493,7 +6493,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Z29</t>
+          <t>ZUZ-LRXD</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Z30</t>
+          <t>ZMZ-MXTD</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -6551,7 +6551,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Z31</t>
+          <t>ZOD-DHJV</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -6580,7 +6580,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Z32</t>
+          <t>ZEK-YCEY</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Z33</t>
+          <t>ZMZ-KWKY</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -6638,7 +6638,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Z34</t>
+          <t>ZOD-JLNI</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -10571,7 +10571,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-01T19:50:39+00:00</t>
+          <t>2026-10-01T20:14:34+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CZ-NACE 2025: rozhodnutí k otázkám z PR #21 (R8–R12)
- R8: změna klasifikace bez počtu odchodů a příchodů – jen počty podle obou verzí, čistá změna,
  hlavní oddíly a „méně než 10“; proměnné klas:* v kontrole dopočtu; stejné pravidlo v kontrolách
  nace_firmy; testy, že z publikovaných čísel nejde dopočítat hodnotu pod 10
- R9: ořez na 1. 1. 2025 jen pro kódy z RES, odvozené kódy se neořezávají (rozhodnutí s důvodem)
- R10, R11: funkce „kód k datu“ povinná před druhým snímkem RES; noční obnova rozhraní po změnách
  z ARES – zapsáno do dalších kroků
- R12: starý pilot (15. 9. 2026) a výstup 10 × CZ063 označené „CZ-NACE 2008, nahrazeno“
  (meta.archiv, vysledek.md, list Přehled, reporty/ukazky/.../ARCHIV.md) a v dokumentaci reportu
- pilot F × Liberecký kraj přepočítaný; text analytika beze změny

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U7RRgPmyDg48516c6s7TrK
</commit_message>
<xml_diff>
--- a/reporty/ukazky/F__CZ051__2026-09-15/priloha.xlsx
+++ b/reporty/ukazky/F__CZ051__2026-09-15/priloha.xlsx
@@ -1,43 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Přehled" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="T01_zakladni" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="T02_srovnani" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="T03_kraje" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="T04_okresy" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="T05_fo_po" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="T06_pravni_forma" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="T07_velikost_fo" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="T08_velikost_po" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="T09_vekova_struktura" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="T13_bench_fo_po" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="T14_bench_pravni_forma" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="T15_bench_velikost_fo" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="T16_bench_velikost_po" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="T17_bench_vekova_struktura" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="T22_ekonomika" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="T23_nahrady" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="T28_model_prepocet" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="T24_model_velikost" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="T25_model_koncentrace" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="T26_sbs_cr" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="T27_model_kontrola" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="T20_mzdy_obor" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="T21_mzdy_aktualni" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="T10_zaniky_po" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="T18_mira_zaniku_po" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="T11_dynamika_csu" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="T12_demografie_cr" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="T19_zjisteni" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Metodika" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="Zdroj a licence" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Přehled" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T01_zakladni" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T02_srovnani" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T03_kraje" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T04_okresy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T05_fo_po" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T06_pravni_forma" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T07_velikost_fo" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T08_velikost_po" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T09_vekova_struktura" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T13_bench_fo_po" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T14_bench_pravni_forma" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T15_bench_velikost_fo" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T16_bench_velikost_po" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T17_bench_vekova_struktura" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T22_ekonomika" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T23_nahrady" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T28_model_prepocet" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T24_model_velikost" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T25_model_koncentrace" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T26_sbs_cr" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T27_model_kontrola" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T20_mzdy_obor" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T21_mzdy_aktualni" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T10_zaniky_po" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T18_mira_zaniku_po" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T11_dynamika_csu" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T12_demografie_cr" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T19_zjisteni" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodika" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zdroj a licence" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -467,468 +467,480 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Obor</t>
+          <t>Archiv</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>F Stavebnictví</t>
+          <t>CZ-NACE 2008, nahrazeno: výstup podle CZ-NACE Rev. 2 (rozhodnutí 5) – archiv. Od 19. 10. 2026 report počítá podle CZ-NACE 2025 (rozhodnutí 15); náhrada: reporty/vystupy/F__CZ051__2026-10-15.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Klasifikace</t>
+          <t>Obor</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CZ-NACE Rev. 2 (klasifikace ČSÚ 80004, sloupec NACE)</t>
+          <t>F Stavebnictví</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Území</t>
+          <t>Klasifikace</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Liberecký kraj (CZ051)</t>
+          <t>CZ-NACE Rev. 2 (klasifikace ČSÚ 80004, sloupec NACE)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Datum snímku RES</t>
+          <t>Území</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>Liberecký kraj (CZ051)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Populace</t>
+          <t>Datum snímku RES</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>registrované ekonomické subjekty bez data zániku (sídlo v území, převažující činnost v oboru)</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Srovnávací kraje (zadal uživatel)</t>
+          <t>Populace</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CZ052, CZ041</t>
+          <t>registrované ekonomické subjekty bez data zániku (sídlo v území, převažující činnost v oboru)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Práh zveřejnění (subjektů)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>10</v>
+          <t>Srovnávací kraje (zadal uživatel)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CZ052, CZ041</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Minimální rozsah reportu (subjektů)</t>
+          <t>Práh zveřejnění (subjektů)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Práh spolehlivosti zařazení (%)</t>
+          <t>Minimální rozsah reportu (subjektů)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Citace</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Zdroj: Český statistický úřad, Registr ekonomických subjektů (RES) – otevřená data, stav k 15. 9. 2026; licence CC BY 4.0 (https://csu.gov.cz/podminky_pro_vyuzivani_a_dalsi_zverejnovani_statistickych_udaju_csu); vlastní výpočet.</t>
-        </is>
+          <t>Práh spolehlivosti zařazení (%)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Citace</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Zdroj: Český statistický úřad, Registr ekonomických subjektů (RES) – otevřená data, stav k 15. 9. 2026; licence CC BY 4.0 (https://csu.gov.cz/podminky_pro_vyuzivani_a_dalsi_zverejnovani_statistickych_udaju_csu); vlastní výpočet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Označení</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Odvozené údaje, nejde o oficiální statistiku ČSÚ.</t>
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Tabulky</t>
-        </is>
-      </c>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>T01_zakladni</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Základní ukazatele</t>
+          <t>Tabulky</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>T02_srovnani</t>
+          <t>T01_zakladni</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Srovnání s ČR a se zadanými kraji</t>
+          <t>Základní ukazatele</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>T03_kraje</t>
+          <t>T02_srovnani</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Pořadí krajů (všech 14)</t>
+          <t>Srovnání s ČR a se zadanými kraji</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>T04_okresy</t>
+          <t>T03_kraje</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Okresy kraje Liberecký kraj</t>
+          <t>Pořadí krajů (všech 14)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>T05_fo_po</t>
+          <t>T04_okresy</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Registrované subjekty podle typu osoby</t>
+          <t>Okresy kraje Liberecký kraj</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>T06_pravni_forma</t>
+          <t>T05_fo_po</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Registrované subjekty podle právní formy (číselník ČSÚ 56)</t>
+          <t>Registrované subjekty podle typu osoby</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>T07_velikost_fo</t>
+          <t>T06_pravni_forma</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Velikostní profil FO podle počtu zaměstnanců (KATPO)</t>
+          <t>Registrované subjekty podle právní formy (číselník ČSÚ 56)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>T08_velikost_po</t>
+          <t>T07_velikost_fo</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Velikostní profil PO podle počtu zaměstnanců (KATPO)</t>
+          <t>Velikostní profil FO podle počtu zaměstnanců (KATPO)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>T09_vekova_struktura</t>
+          <t>T08_velikost_po</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Věková struktura existujících subjektů</t>
+          <t>Velikostní profil PO podle počtu zaměstnanců (KATPO)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>T13_bench_fo_po</t>
+          <t>T09_vekova_struktura</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Typ osoby – srovnání s ČR a se srovnávacími kraji (podíl, %)</t>
+          <t>Věková struktura existujících subjektů</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>T14_bench_pravni_forma</t>
+          <t>T13_bench_fo_po</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Právní forma – srovnání s ČR a se srovnávacími kraji (podíl z celku, %)</t>
+          <t>Typ osoby – srovnání s ČR a se srovnávacími kraji (podíl, %)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>T15_bench_velikost_fo</t>
+          <t>T14_bench_pravni_forma</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Velikostní profil FO – srovnání s ČR a se srovnávacími kraji (podíl z FO, %)</t>
+          <t>Právní forma – srovnání s ČR a se srovnávacími kraji (podíl z celku, %)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>T16_bench_velikost_po</t>
+          <t>T15_bench_velikost_fo</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Velikostní profil PO – srovnání s ČR a se srovnávacími kraji (podíl z PO, %)</t>
+          <t>Velikostní profil FO – srovnání s ČR a se srovnávacími kraji (podíl z FO, %)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>T17_bench_vekova_struktura</t>
+          <t>T16_bench_velikost_po</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Věková struktura existujících subjektů – srovnání s ČR a se srovnávacími kraji (podíl, %)</t>
+          <t>Velikostní profil PO – srovnání s ČR a se srovnávacími kraji (podíl z PO, %)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>T22_ekonomika</t>
+          <t>T17_bench_vekova_struktura</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Hrubá přidaná hodnota, zaměstnanost a produktivita – kraje a ČR (Eurostat, regionální účty) – Stavebnictví (F)</t>
+          <t>Věková struktura existujících subjektů – srovnání s ČR a se srovnávacími kraji (podíl, %)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>T23_nahrady</t>
+          <t>T22_ekonomika</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Náhrady zaměstnancům a hrubá přidaná hodnota – regiony soudržnosti (Eurostat) – Stavebnictví (F)</t>
+          <t>Hrubá přidaná hodnota, zaměstnanost a produktivita – kraje a ČR (Eurostat, regionální účty) – Stavebnictví (F)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>T28_model_prepocet</t>
+          <t>T23_nahrady</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Přepočet přidané hodnoty na úroveň statistiky podniků (vstup modelu) – Liberecký kraj, 2024</t>
+          <t>Náhrady zaměstnancům a hrubá přidaná hodnota – regiony soudržnosti (Eurostat) – Stavebnictví (F)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>T24_model_velikost</t>
+          <t>T28_model_prepocet</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Modelový odhad: přidaná hodnota a obrat oboru podle velikosti subjektů – Liberecký kraj, 2024</t>
+          <t>Přepočet přidané hodnoty na úroveň statistiky podniků (vstup modelu) – Liberecký kraj, 2024</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>T25_model_koncentrace</t>
+          <t>T24_model_velikost</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Modelový odhad: koncentrace – podíl subjektů s 10+ a 50+ zaměstnanými osobami – Liberecký kraj, 2024</t>
+          <t>Modelový odhad: přidaná hodnota a obrat oboru podle velikosti subjektů – Liberecký kraj, 2024</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>T26_sbs_cr</t>
+          <t>T25_model_koncentrace</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Statistika podniků za ČR podle velikosti: typický obrat a marže (fakt za ČR, Eurostat SBS) – sekce F, 2024</t>
+          <t>Modelový odhad: koncentrace – podíl subjektů s 10+ a 50+ zaměstnanými osobami – Liberecký kraj, 2024</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>T27_model_kontrola</t>
+          <t>T26_sbs_cr</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Kontrola konzistence: model použitý na celou ČR proti statistice podniků (SBS) – sekce F, 2024</t>
+          <t>Statistika podniků za ČR podle velikosti: typický obrat a marže (fakt za ČR, Eurostat SBS) – sekce F, 2024</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>T20_mzdy_obor</t>
+          <t>T27_model_kontrola</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Zaměstnanci a průměrné mzdy v oboru – kraje a ČR (ČSÚ, roční zjišťování)</t>
+          <t>Kontrola konzistence: model použitý na celou ČR proti statistice podniků (SBS) – sekce F, 2024</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>T21_mzdy_aktualni</t>
+          <t>T20_mzdy_obor</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Zaměstnanci a průměrné mzdy – novější roky v nejbližších publikovaných úrovních (ČSÚ, čtvrtletní zjišťování)</t>
+          <t>Zaměstnanci a průměrné mzdy v oboru – kraje a ČR (ČSÚ, roční zjišťování)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>T10_zaniky_po</t>
+          <t>T21_mzdy_aktualni</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Zaniklé právnické osoby v oboru a území podle roku zániku (RES, od 2023)</t>
+          <t>Zaměstnanci a průměrné mzdy – novější roky v nejbližších publikovaných úrovních (ČSÚ, čtvrtletní zjišťování)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>T18_mira_zaniku_po</t>
+          <t>T10_zaniky_po</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Míra zániku právnických osob v oboru (RES, 2023–2026)</t>
+          <t>Zaniklé právnické osoby v oboru a území podle roku zániku (RES, od 2023)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>T11_dynamika_csu</t>
+          <t>T18_mira_zaniku_po</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Vznik a zánik ekonomických subjektů v území – všechny obory (ČSÚ, RES05)</t>
+          <t>Míra zániku právnických osob v oboru (RES, 2023–2026)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>T12_demografie_cr</t>
+          <t>T11_dynamika_csu</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Demografie podniků v ČR – kontext (ČSÚ, RESDP00; jednotka podnik)</t>
+          <t>Vznik a zánik ekonomických subjektů v území – všechny obory (ČSÚ, RES05)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>T12_demografie_cr</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Demografie podniků v ČR – kontext (ČSÚ, RESDP00; jednotka podnik)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>T19_zjisteni</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>Zjištění detektoru (seřazeno podle síly)</t>
         </is>
@@ -9786,7 +9798,6 @@
           <t>ČSÚ DataStat – tabulka v tomto členění neexistuje (RES05 jen území × FO/PO; RES06 registrace a RESDP00 demografie podniků jen za ČR podle odvětví)</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>Nelze naplnit.</t>

</xml_diff>